<commit_message>
Atualização dos scripts - troca de máquina
</commit_message>
<xml_diff>
--- a/DE-PARA.xlsx
+++ b/DE-PARA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Importacoes\Franqueadoras\LASER ROSA\Scripts\teste\entrada\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\geinfo\Desktop\Importações\Franqueadoras\Laser Rosa\Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF3F951-B701-4F49-AA54-21E286510054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F7A51A-D38E-4833-B461-3A3B8318CDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15660" yWindow="-5715" windowWidth="15045" windowHeight="9915" xr2:uid="{98C53999-9006-4998-8C04-936FF5F0754C}"/>
+    <workbookView xWindow="-14685" yWindow="9915" windowWidth="13125" windowHeight="11100" activeTab="3" xr2:uid="{98C53999-9006-4998-8C04-936FF5F0754C}"/>
   </bookViews>
   <sheets>
     <sheet name="serv" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="sala" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">serv!$L$1:$L$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">serv!$A$1:$A$332</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="206">
   <si>
     <t>Item</t>
   </si>
@@ -646,13 +646,16 @@
   </si>
   <si>
     <t>Código</t>
+  </si>
+  <si>
+    <t>VIRILHA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -690,6 +693,12 @@
       <color rgb="FF334155"/>
       <name val="Manrope"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -711,7 +720,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -723,6 +732,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1038,14 +1048,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61B7A6AF-9F82-47E8-9A9F-1598495EF00A}">
   <dimension ref="A1:H332"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="3" width="9.28515625" customWidth="1"/>
-    <col min="4" max="5" width="6.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="2" max="3" width="9.33203125" customWidth="1"/>
+    <col min="4" max="5" width="6.6640625" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
     <col min="7" max="8" width="10" customWidth="1"/>
-    <col min="9" max="10" width="6.5703125" customWidth="1"/>
+    <col min="9" max="10" width="6.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4286,8 +4296,12 @@
       </c>
     </row>
     <row r="332" spans="1:2">
-      <c r="A332" s="2"/>
-      <c r="B332" s="2"/>
+      <c r="A332" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B332" s="7">
+        <v>33421041</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -4297,7 +4311,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4ABB8EAC-315B-4DBB-AECF-8BB0E4FCF5CB}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -4360,7 +4374,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0874ACBA-0099-40FC-A443-6E4A9AF19F09}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
@@ -4410,7 +4424,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAB741D8-969F-4ABB-9050-2F2E4FAE8ACB}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">

</xml_diff>